<commit_message>
added websocket connection, telemetry view and reorganized svelte lib
</commit_message>
<xml_diff>
--- a/sw/firmware/OBDII-PIDs.xlsx
+++ b/sw/firmware/OBDII-PIDs.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jpojsl\Desktop\code\ESP\CAN-Sniffer\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kubai\Documents\CAN-Sniffer\sw\firmware\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E86D5EEA-E25B-44B2-A250-C89F6E62D0F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA833BB2-29C9-4D0D-ADCF-C0CBA790C86C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{429A65A5-501F-4DDC-877A-2B2A6BFACDF8}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{429A65A5-501F-4DDC-877A-2B2A6BFACDF8}"/>
   </bookViews>
   <sheets>
-    <sheet name="obd2-pid-table-service-01" sheetId="2" r:id="rId1"/>
-    <sheet name="Sheet1" sheetId="1" r:id="rId2"/>
+    <sheet name="obd2-pid" sheetId="2" r:id="rId1"/>
+    <sheet name="usd-dids" sheetId="1" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="ExternalData_1" localSheetId="0" hidden="1">'obd2-pid-table-service-01'!$A$1:$N$206</definedName>
+    <definedName name="ExternalData_1" localSheetId="0" hidden="1">'obd2-pid'!$A$1:$N$206</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -31,8 +31,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -48,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1654" uniqueCount="633">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1725" uniqueCount="682">
   <si>
     <t>PID (dec)</t>
   </si>
@@ -1947,13 +1945,160 @@
   </si>
   <si>
     <t>PIDs supported [C1 - E0]</t>
+  </si>
+  <si>
+    <t>Car</t>
+  </si>
+  <si>
+    <t>Module Name</t>
+  </si>
+  <si>
+    <t>Module ID</t>
+  </si>
+  <si>
+    <t>Example Request</t>
+  </si>
+  <si>
+    <t>Example Response</t>
+  </si>
+  <si>
+    <t>Bit S|L</t>
+  </si>
+  <si>
+    <t>Instruments</t>
+  </si>
+  <si>
+    <t>0x714</t>
+  </si>
+  <si>
+    <t>m</t>
+  </si>
+  <si>
+    <t>05 62 22 03 3A AA</t>
+  </si>
+  <si>
+    <t>32 | 16</t>
+  </si>
+  <si>
+    <t>Fuel Level</t>
+  </si>
+  <si>
+    <t>L</t>
+  </si>
+  <si>
+    <t>04 62 22 06 0C</t>
+  </si>
+  <si>
+    <t>32 | 8</t>
+  </si>
+  <si>
+    <t>BCM</t>
+  </si>
+  <si>
+    <t>0x70C</t>
+  </si>
+  <si>
+    <t>Turn Signals</t>
+  </si>
+  <si>
+    <t>Enum</t>
+  </si>
+  <si>
+    <t>03 22 1F 00</t>
+  </si>
+  <si>
+    <t>04 62 1F 00 01</t>
+  </si>
+  <si>
+    <t>High Beam</t>
+  </si>
+  <si>
+    <t>Bit</t>
+  </si>
+  <si>
+    <t>03 22 1F 02</t>
+  </si>
+  <si>
+    <t>04 62 1F 02 01</t>
+  </si>
+  <si>
+    <t>Doors/Lids</t>
+  </si>
+  <si>
+    <t>Mask</t>
+  </si>
+  <si>
+    <t>03 22 1F 05</t>
+  </si>
+  <si>
+    <t>04 62 1F 05 11</t>
+  </si>
+  <si>
+    <t>HVAC</t>
+  </si>
+  <si>
+    <t>0x746</t>
+  </si>
+  <si>
+    <t>Interior Temp</t>
+  </si>
+  <si>
+    <t>°C</t>
+  </si>
+  <si>
+    <t>05 62 26 13 00 6B</t>
+  </si>
+  <si>
+    <t>Golf mk6</t>
+  </si>
+  <si>
+    <t>0x2203</t>
+  </si>
+  <si>
+    <t>0x2206</t>
+  </si>
+  <si>
+    <t>0x1F00</t>
+  </si>
+  <si>
+    <t>0x1F02</t>
+  </si>
+  <si>
+    <t>0x1F05</t>
+  </si>
+  <si>
+    <t>0x2613</t>
+  </si>
+  <si>
+    <t>03 22 22 03</t>
+  </si>
+  <si>
+    <t>03 22 22 06</t>
+  </si>
+  <si>
+    <t>03 22 26 13</t>
+  </si>
+  <si>
+    <t>Sloupec1</t>
+  </si>
+  <si>
+    <t>Result = ((A * 256) + B) * 10</t>
+  </si>
+  <si>
+    <t>Result = ((A * 256) + B) * 0.1</t>
+  </si>
+  <si>
+    <t>Passenger door | Rear Left | Rear right | Trunk | Hood</t>
+  </si>
+  <si>
+    <t>https://gemini.google.com/share/4034399b676c</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1961,6 +2106,19 @@
       <family val="2"/>
       <charset val="238"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <charset val="238"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1983,13 +2141,26 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normální" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="8">
+  <dxfs count="11">
+    <dxf>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
@@ -2055,19 +2226,40 @@
   <autoFilter ref="A1:N206" xr:uid="{2DFB9FBA-2467-4995-B604-1918573FF354}"/>
   <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{FFCF6DEB-2999-481B-A490-10AE159DCC24}" uniqueName="1" name="PID (dec)" queryTableFieldId="1"/>
-    <tableColumn id="2" xr3:uid="{AB89E74A-2973-45B7-B1E2-266DEEF6796D}" uniqueName="2" name="PID (hex)" queryTableFieldId="2" dataDxfId="7"/>
-    <tableColumn id="3" xr3:uid="{B9046B97-C173-4F4A-B9B8-9A20A8A31CC7}" uniqueName="3" name="Name (short)" queryTableFieldId="3" dataDxfId="6"/>
-    <tableColumn id="4" xr3:uid="{C84322B4-4BAC-48F9-ADF3-8E6EC3A6C2F1}" uniqueName="4" name="Name" queryTableFieldId="4" dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{AB89E74A-2973-45B7-B1E2-266DEEF6796D}" uniqueName="2" name="PID (hex)" queryTableFieldId="2" dataDxfId="10"/>
+    <tableColumn id="3" xr3:uid="{B9046B97-C173-4F4A-B9B8-9A20A8A31CC7}" uniqueName="3" name="Name (short)" queryTableFieldId="3" dataDxfId="9"/>
+    <tableColumn id="4" xr3:uid="{C84322B4-4BAC-48F9-ADF3-8E6EC3A6C2F1}" uniqueName="4" name="Name" queryTableFieldId="4" dataDxfId="8"/>
     <tableColumn id="5" xr3:uid="{42B6162C-8A22-462D-AABF-21B568F0DDF8}" uniqueName="5" name="Bit start" queryTableFieldId="5"/>
     <tableColumn id="6" xr3:uid="{80E67AE3-544B-4C77-89C3-BADF48DC5E53}" uniqueName="6" name="Bit length" queryTableFieldId="6"/>
-    <tableColumn id="7" xr3:uid="{995B76F1-4959-4136-A167-BC15E0288327}" uniqueName="7" name="Scale" queryTableFieldId="7" dataDxfId="4"/>
+    <tableColumn id="7" xr3:uid="{995B76F1-4959-4136-A167-BC15E0288327}" uniqueName="7" name="Scale" queryTableFieldId="7" dataDxfId="7"/>
     <tableColumn id="8" xr3:uid="{C053313C-ACEF-47A9-B1D0-440EFB6DF09F}" uniqueName="8" name="Offset" queryTableFieldId="8"/>
     <tableColumn id="9" xr3:uid="{22C07886-330C-4B5F-BB60-7CE62692BFC7}" uniqueName="9" name="Min" queryTableFieldId="9"/>
     <tableColumn id="10" xr3:uid="{4C9615AF-4938-4DB9-95E3-2B787B51D1AE}" uniqueName="10" name="Max" queryTableFieldId="10"/>
-    <tableColumn id="11" xr3:uid="{545246C6-CF9F-4786-85E8-A85CF2E8415D}" uniqueName="11" name="Unit" queryTableFieldId="11" dataDxfId="3"/>
-    <tableColumn id="12" xr3:uid="{24D167A7-F54F-41B8-AAC2-446225857EDC}" uniqueName="12" name="Scale (short)" queryTableFieldId="12" dataDxfId="2"/>
-    <tableColumn id="13" xr3:uid="{3E020E81-A633-4F19-99B7-DAD9A8908E1B}" uniqueName="13" name="Min | Max" queryTableFieldId="13" dataDxfId="1"/>
-    <tableColumn id="14" xr3:uid="{4DEF838A-ED5B-402D-AF91-67770AA65818}" uniqueName="14" name="Bit start | length" queryTableFieldId="14" dataDxfId="0"/>
+    <tableColumn id="11" xr3:uid="{545246C6-CF9F-4786-85E8-A85CF2E8415D}" uniqueName="11" name="Unit" queryTableFieldId="11" dataDxfId="6"/>
+    <tableColumn id="12" xr3:uid="{24D167A7-F54F-41B8-AAC2-446225857EDC}" uniqueName="12" name="Scale (short)" queryTableFieldId="12" dataDxfId="5"/>
+    <tableColumn id="13" xr3:uid="{3E020E81-A633-4F19-99B7-DAD9A8908E1B}" uniqueName="13" name="Min | Max" queryTableFieldId="13" dataDxfId="4"/>
+    <tableColumn id="14" xr3:uid="{4DEF838A-ED5B-402D-AF91-67770AA65818}" uniqueName="14" name="Bit start | length" queryTableFieldId="14" dataDxfId="3"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{4F04E350-6D47-4E09-A10B-E6A8E1D51955}" name="Tabulka2" displayName="Tabulka2" ref="A1:L7" totalsRowShown="0">
+  <autoFilter ref="A1:L7" xr:uid="{4F04E350-6D47-4E09-A10B-E6A8E1D51955}"/>
+  <tableColumns count="12">
+    <tableColumn id="1" xr3:uid="{984946A5-A725-4CB2-BED2-DAC7593D2235}" name="Car"/>
+    <tableColumn id="2" xr3:uid="{9D892733-4D76-4C99-8DC4-07953415758A}" name="Module Name"/>
+    <tableColumn id="3" xr3:uid="{10BD86BD-0BAD-4B7E-90DB-2D0150792BAC}" name="Module ID"/>
+    <tableColumn id="4" xr3:uid="{CBE9C179-B488-45FE-A5E1-4BFF06D0AC9B}" name="PID (hex)" dataDxfId="2"/>
+    <tableColumn id="5" xr3:uid="{7495D6DB-4DDB-4BCC-9CA2-8C0F6F941688}" name="Name"/>
+    <tableColumn id="6" xr3:uid="{BAEDB00A-525C-441C-96B4-8B0C3E417767}" name="Scale"/>
+    <tableColumn id="7" xr3:uid="{7F534183-0C16-42F7-9F39-95E49B7E9C7D}" name="Offset"/>
+    <tableColumn id="8" xr3:uid="{7DA35E7A-7618-4727-862A-7FEF7D2384DA}" name="Unit"/>
+    <tableColumn id="9" xr3:uid="{6420B9FA-17D6-4BDD-905E-B24C9FFECF0B}" name="Example Request" dataDxfId="1"/>
+    <tableColumn id="10" xr3:uid="{AF2DE9E7-F7D7-40A7-B409-1C9D7BC25D21}" name="Example Response" dataDxfId="0"/>
+    <tableColumn id="11" xr3:uid="{29F6CD0E-77A6-469F-94F0-37C29C2492CF}" name="Bit S|L"/>
+    <tableColumn id="12" xr3:uid="{DF261B1A-8F21-48FD-902C-7E2E39B9973C}" name="Sloupec1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2391,24 +2583,24 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{648A89BD-0A8A-40CB-A70D-EE942ADB2874}">
   <dimension ref="A1:N206"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="2" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="30.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="36.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="11.625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="30.375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="36.625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.25" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.75" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="9" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="6.75" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="7" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.25" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="14.75" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.75" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="18" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2452,7 +2644,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14">
       <c r="A2">
         <v>0</v>
       </c>
@@ -2490,7 +2682,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14">
       <c r="A3">
         <v>1</v>
       </c>
@@ -2528,7 +2720,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14">
       <c r="A4">
         <v>2</v>
       </c>
@@ -2566,7 +2758,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:14">
       <c r="A5">
         <v>3</v>
       </c>
@@ -2604,7 +2796,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14">
       <c r="A6">
         <v>4</v>
       </c>
@@ -2648,7 +2840,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:14">
       <c r="A7">
         <v>5</v>
       </c>
@@ -2692,7 +2884,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:14">
       <c r="A8">
         <v>6</v>
       </c>
@@ -2736,7 +2928,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14">
       <c r="A9">
         <v>7</v>
       </c>
@@ -2780,7 +2972,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:14">
       <c r="A10">
         <v>8</v>
       </c>
@@ -2824,7 +3016,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:14">
       <c r="A11">
         <v>9</v>
       </c>
@@ -2868,7 +3060,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:14">
       <c r="A12">
         <v>10</v>
       </c>
@@ -2912,7 +3104,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:14">
       <c r="A13">
         <v>11</v>
       </c>
@@ -2956,7 +3148,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:14">
       <c r="A14">
         <v>12</v>
       </c>
@@ -3000,7 +3192,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:14">
       <c r="A15">
         <v>13</v>
       </c>
@@ -3044,7 +3236,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:14">
       <c r="A16">
         <v>14</v>
       </c>
@@ -3088,7 +3280,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:14">
       <c r="A17">
         <v>15</v>
       </c>
@@ -3132,7 +3324,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:14">
       <c r="A18">
         <v>16</v>
       </c>
@@ -3176,7 +3368,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:14">
       <c r="A19">
         <v>17</v>
       </c>
@@ -3220,7 +3412,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:14">
       <c r="A20">
         <v>18</v>
       </c>
@@ -3258,7 +3450,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:14">
       <c r="A21">
         <v>19</v>
       </c>
@@ -3287,7 +3479,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:14">
       <c r="A22">
         <v>20</v>
       </c>
@@ -3331,7 +3523,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:14">
       <c r="B23" t="s">
         <v>19</v>
       </c>
@@ -3372,7 +3564,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:14">
       <c r="A24">
         <v>21</v>
       </c>
@@ -3416,7 +3608,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:14">
       <c r="B25" t="s">
         <v>19</v>
       </c>
@@ -3457,7 +3649,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:14">
       <c r="A26">
         <v>22</v>
       </c>
@@ -3501,7 +3693,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:14">
       <c r="B27" t="s">
         <v>19</v>
       </c>
@@ -3542,7 +3734,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:14">
       <c r="A28">
         <v>23</v>
       </c>
@@ -3586,7 +3778,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:14">
       <c r="B29" t="s">
         <v>19</v>
       </c>
@@ -3627,7 +3819,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:14">
       <c r="A30">
         <v>24</v>
       </c>
@@ -3671,7 +3863,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:14">
       <c r="B31" t="s">
         <v>19</v>
       </c>
@@ -3712,7 +3904,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:14">
       <c r="A32">
         <v>25</v>
       </c>
@@ -3756,7 +3948,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:14">
       <c r="B33" t="s">
         <v>19</v>
       </c>
@@ -3797,7 +3989,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:14">
       <c r="A34">
         <v>26</v>
       </c>
@@ -3841,7 +4033,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:14">
       <c r="B35" t="s">
         <v>19</v>
       </c>
@@ -3882,7 +4074,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:14">
       <c r="A36">
         <v>27</v>
       </c>
@@ -3926,7 +4118,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:14">
       <c r="B37" t="s">
         <v>19</v>
       </c>
@@ -3967,7 +4159,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="38" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:14">
       <c r="A38">
         <v>28</v>
       </c>
@@ -4005,7 +4197,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="39" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:14">
       <c r="A39">
         <v>29</v>
       </c>
@@ -4034,7 +4226,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="40" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:14">
       <c r="A40">
         <v>30</v>
       </c>
@@ -4063,7 +4255,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="41" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:14">
       <c r="A41">
         <v>31</v>
       </c>
@@ -4107,7 +4299,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="42" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:14">
       <c r="A42">
         <v>32</v>
       </c>
@@ -4145,7 +4337,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="43" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:14">
       <c r="A43">
         <v>33</v>
       </c>
@@ -4189,7 +4381,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="44" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:14">
       <c r="A44">
         <v>34</v>
       </c>
@@ -4233,7 +4425,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="45" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:14">
       <c r="A45">
         <v>35</v>
       </c>
@@ -4277,7 +4469,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="46" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:14">
       <c r="A46">
         <v>36</v>
       </c>
@@ -4321,7 +4513,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="47" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:14">
       <c r="B47" t="s">
         <v>19</v>
       </c>
@@ -4362,7 +4554,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="48" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:14">
       <c r="A48">
         <v>37</v>
       </c>
@@ -4406,7 +4598,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="49" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:14">
       <c r="B49" t="s">
         <v>19</v>
       </c>
@@ -4447,7 +4639,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="50" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:14">
       <c r="A50">
         <v>38</v>
       </c>
@@ -4491,7 +4683,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="51" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:14">
       <c r="B51" t="s">
         <v>19</v>
       </c>
@@ -4532,7 +4724,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="52" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:14">
       <c r="A52">
         <v>39</v>
       </c>
@@ -4576,7 +4768,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="53" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:14">
       <c r="B53" t="s">
         <v>19</v>
       </c>
@@ -4617,7 +4809,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="54" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:14">
       <c r="A54">
         <v>40</v>
       </c>
@@ -4661,7 +4853,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="55" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:14">
       <c r="B55" t="s">
         <v>19</v>
       </c>
@@ -4702,7 +4894,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="56" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:14">
       <c r="A56">
         <v>41</v>
       </c>
@@ -4746,7 +4938,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="57" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:14">
       <c r="B57" t="s">
         <v>19</v>
       </c>
@@ -4787,7 +4979,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="58" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:14">
       <c r="A58">
         <v>42</v>
       </c>
@@ -4831,7 +5023,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="59" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:14">
       <c r="B59" t="s">
         <v>19</v>
       </c>
@@ -4872,7 +5064,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="60" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:14">
       <c r="A60">
         <v>43</v>
       </c>
@@ -4916,7 +5108,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="61" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:14">
       <c r="B61" t="s">
         <v>19</v>
       </c>
@@ -4957,7 +5149,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="62" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:14">
       <c r="A62">
         <v>44</v>
       </c>
@@ -5001,7 +5193,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="63" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:14">
       <c r="A63">
         <v>45</v>
       </c>
@@ -5045,7 +5237,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="64" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:14">
       <c r="A64">
         <v>46</v>
       </c>
@@ -5089,7 +5281,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="65" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:14">
       <c r="A65">
         <v>47</v>
       </c>
@@ -5133,7 +5325,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="66" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:14">
       <c r="A66">
         <v>48</v>
       </c>
@@ -5177,7 +5369,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="67" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:14">
       <c r="A67">
         <v>49</v>
       </c>
@@ -5221,7 +5413,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="68" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:14">
       <c r="A68">
         <v>50</v>
       </c>
@@ -5265,7 +5457,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="69" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:14">
       <c r="A69">
         <v>51</v>
       </c>
@@ -5309,7 +5501,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="70" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:14">
       <c r="A70">
         <v>52</v>
       </c>
@@ -5353,7 +5545,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="71" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:14">
       <c r="B71" t="s">
         <v>19</v>
       </c>
@@ -5394,7 +5586,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="72" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:14">
       <c r="A72">
         <v>53</v>
       </c>
@@ -5438,7 +5630,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="73" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:14">
       <c r="B73" t="s">
         <v>19</v>
       </c>
@@ -5479,7 +5671,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="74" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:14">
       <c r="A74">
         <v>54</v>
       </c>
@@ -5523,7 +5715,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="75" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:14">
       <c r="B75" t="s">
         <v>19</v>
       </c>
@@ -5564,7 +5756,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="76" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:14">
       <c r="A76">
         <v>55</v>
       </c>
@@ -5608,7 +5800,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="77" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:14">
       <c r="B77" t="s">
         <v>19</v>
       </c>
@@ -5649,7 +5841,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="78" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:14">
       <c r="A78">
         <v>56</v>
       </c>
@@ -5693,7 +5885,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="79" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:14">
       <c r="B79" t="s">
         <v>19</v>
       </c>
@@ -5734,7 +5926,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="80" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:14">
       <c r="A80">
         <v>57</v>
       </c>
@@ -5778,7 +5970,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="81" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:14">
       <c r="B81" t="s">
         <v>19</v>
       </c>
@@ -5819,7 +6011,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="82" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:14">
       <c r="A82">
         <v>58</v>
       </c>
@@ -5863,7 +6055,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="83" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:14">
       <c r="B83" t="s">
         <v>19</v>
       </c>
@@ -5904,7 +6096,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="84" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:14">
       <c r="A84">
         <v>59</v>
       </c>
@@ -5948,7 +6140,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="85" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:14">
       <c r="B85" t="s">
         <v>19</v>
       </c>
@@ -5989,7 +6181,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="86" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:14">
       <c r="A86">
         <v>60</v>
       </c>
@@ -6033,7 +6225,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="87" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:14">
       <c r="A87">
         <v>61</v>
       </c>
@@ -6077,7 +6269,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="88" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:14">
       <c r="A88">
         <v>62</v>
       </c>
@@ -6121,7 +6313,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="89" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:14">
       <c r="A89">
         <v>63</v>
       </c>
@@ -6165,7 +6357,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="90" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:14">
       <c r="A90">
         <v>64</v>
       </c>
@@ -6203,7 +6395,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="91" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:14">
       <c r="A91">
         <v>65</v>
       </c>
@@ -6241,7 +6433,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="92" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:14">
       <c r="A92">
         <v>66</v>
       </c>
@@ -6285,7 +6477,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="93" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:14">
       <c r="A93">
         <v>67</v>
       </c>
@@ -6329,7 +6521,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="94" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:14">
       <c r="A94">
         <v>68</v>
       </c>
@@ -6373,7 +6565,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="95" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:14">
       <c r="A95">
         <v>69</v>
       </c>
@@ -6417,7 +6609,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="96" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:14">
       <c r="A96">
         <v>70</v>
       </c>
@@ -6461,7 +6653,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="97" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:14">
       <c r="A97">
         <v>71</v>
       </c>
@@ -6505,7 +6697,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="98" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:14">
       <c r="A98">
         <v>72</v>
       </c>
@@ -6549,7 +6741,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="99" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:14">
       <c r="A99">
         <v>73</v>
       </c>
@@ -6593,7 +6785,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="100" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:14">
       <c r="A100">
         <v>74</v>
       </c>
@@ -6637,7 +6829,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="101" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:14">
       <c r="A101">
         <v>75</v>
       </c>
@@ -6681,7 +6873,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="102" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:14">
       <c r="A102">
         <v>76</v>
       </c>
@@ -6725,7 +6917,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="103" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:14">
       <c r="A103">
         <v>77</v>
       </c>
@@ -6769,7 +6961,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="104" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:14">
       <c r="A104">
         <v>78</v>
       </c>
@@ -6813,7 +7005,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="105" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:14">
       <c r="A105">
         <v>79</v>
       </c>
@@ -6857,7 +7049,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="106" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:14">
       <c r="B106" t="s">
         <v>19</v>
       </c>
@@ -6898,7 +7090,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="107" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:14">
       <c r="B107" t="s">
         <v>19</v>
       </c>
@@ -6939,7 +7131,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="108" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:14">
       <c r="B108" t="s">
         <v>19</v>
       </c>
@@ -6980,7 +7172,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="109" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:14">
       <c r="A109">
         <v>80</v>
       </c>
@@ -7024,7 +7216,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="110" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:14">
       <c r="A110">
         <v>81</v>
       </c>
@@ -7062,7 +7254,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="111" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:14">
       <c r="A111">
         <v>82</v>
       </c>
@@ -7106,7 +7298,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="112" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:14">
       <c r="A112">
         <v>83</v>
       </c>
@@ -7150,7 +7342,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="113" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:14">
       <c r="A113">
         <v>84</v>
       </c>
@@ -7194,7 +7386,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="114" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:14">
       <c r="A114">
         <v>85</v>
       </c>
@@ -7238,7 +7430,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="115" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:14">
       <c r="B115" t="s">
         <v>19</v>
       </c>
@@ -7279,7 +7471,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="116" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:14">
       <c r="A116">
         <v>86</v>
       </c>
@@ -7323,7 +7515,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="117" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:14">
       <c r="B117" t="s">
         <v>19</v>
       </c>
@@ -7364,7 +7556,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="118" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:14">
       <c r="A118">
         <v>87</v>
       </c>
@@ -7408,7 +7600,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="119" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:14">
       <c r="B119" t="s">
         <v>19</v>
       </c>
@@ -7449,7 +7641,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="120" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:14">
       <c r="A120">
         <v>88</v>
       </c>
@@ -7493,7 +7685,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="121" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:14">
       <c r="B121" t="s">
         <v>19</v>
       </c>
@@ -7534,7 +7726,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="122" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:14">
       <c r="A122">
         <v>89</v>
       </c>
@@ -7578,7 +7770,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="123" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:14">
       <c r="A123">
         <v>90</v>
       </c>
@@ -7622,7 +7814,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="124" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:14">
       <c r="A124">
         <v>91</v>
       </c>
@@ -7666,7 +7858,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="125" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:14">
       <c r="A125">
         <v>92</v>
       </c>
@@ -7710,7 +7902,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="126" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:14">
       <c r="A126">
         <v>93</v>
       </c>
@@ -7754,7 +7946,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="127" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:14">
       <c r="A127">
         <v>94</v>
       </c>
@@ -7798,7 +7990,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="128" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:14">
       <c r="A128">
         <v>95</v>
       </c>
@@ -7836,7 +8028,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="129" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:14">
       <c r="A129">
         <v>96</v>
       </c>
@@ -7874,7 +8066,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="130" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:14">
       <c r="A130">
         <v>97</v>
       </c>
@@ -7918,7 +8110,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="131" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:14">
       <c r="A131">
         <v>98</v>
       </c>
@@ -7962,7 +8154,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="132" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:14">
       <c r="A132">
         <v>99</v>
       </c>
@@ -8006,7 +8198,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="133" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:14">
       <c r="A133">
         <v>100</v>
       </c>
@@ -8050,7 +8242,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="134" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:14">
       <c r="B134" t="s">
         <v>19</v>
       </c>
@@ -8091,7 +8283,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="135" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:14">
       <c r="B135" t="s">
         <v>19</v>
       </c>
@@ -8132,7 +8324,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="136" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:14">
       <c r="B136" t="s">
         <v>19</v>
       </c>
@@ -8173,7 +8365,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="137" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:14">
       <c r="B137" t="s">
         <v>19</v>
       </c>
@@ -8214,7 +8406,7 @@
         <v>430</v>
       </c>
     </row>
-    <row r="138" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:14">
       <c r="A138">
         <v>101</v>
       </c>
@@ -8252,7 +8444,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="139" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:14">
       <c r="A139">
         <v>102</v>
       </c>
@@ -8296,7 +8488,7 @@
         <v>440</v>
       </c>
     </row>
-    <row r="140" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:14">
       <c r="B140" t="s">
         <v>19</v>
       </c>
@@ -8337,7 +8529,7 @@
         <v>443</v>
       </c>
     </row>
-    <row r="141" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:14">
       <c r="A141">
         <v>103</v>
       </c>
@@ -8381,7 +8573,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="142" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:14">
       <c r="B142" t="s">
         <v>19</v>
       </c>
@@ -8422,7 +8614,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="143" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:14">
       <c r="A143">
         <v>104</v>
       </c>
@@ -8466,7 +8658,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="144" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:14">
       <c r="B144" t="s">
         <v>19</v>
       </c>
@@ -8507,7 +8699,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="145" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:14">
       <c r="A145">
         <v>105</v>
       </c>
@@ -8536,7 +8728,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="146" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:14">
       <c r="A146">
         <v>106</v>
       </c>
@@ -8565,7 +8757,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="147" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:14">
       <c r="A147">
         <v>107</v>
       </c>
@@ -8594,7 +8786,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="148" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:14">
       <c r="A148">
         <v>108</v>
       </c>
@@ -8623,7 +8815,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="149" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:14">
       <c r="A149">
         <v>109</v>
       </c>
@@ -8652,7 +8844,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="150" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:14">
       <c r="A150">
         <v>110</v>
       </c>
@@ -8681,7 +8873,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="151" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:14">
       <c r="A151">
         <v>111</v>
       </c>
@@ -8710,7 +8902,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="152" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:14">
       <c r="A152">
         <v>112</v>
       </c>
@@ -8739,7 +8931,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="153" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:14">
       <c r="A153">
         <v>113</v>
       </c>
@@ -8768,7 +8960,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="154" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:14">
       <c r="A154">
         <v>114</v>
       </c>
@@ -8797,7 +8989,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="155" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:14">
       <c r="A155">
         <v>115</v>
       </c>
@@ -8826,7 +9018,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="156" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:14">
       <c r="A156">
         <v>116</v>
       </c>
@@ -8855,7 +9047,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="157" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:14">
       <c r="A157">
         <v>117</v>
       </c>
@@ -8884,7 +9076,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="158" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:14">
       <c r="A158">
         <v>118</v>
       </c>
@@ -8913,7 +9105,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="159" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:14">
       <c r="A159">
         <v>119</v>
       </c>
@@ -8942,7 +9134,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="160" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:14">
       <c r="A160">
         <v>120</v>
       </c>
@@ -8971,7 +9163,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="161" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:14">
       <c r="A161">
         <v>121</v>
       </c>
@@ -9000,7 +9192,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="162" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:14">
       <c r="A162">
         <v>122</v>
       </c>
@@ -9029,7 +9221,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="163" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:14">
       <c r="A163">
         <v>123</v>
       </c>
@@ -9058,7 +9250,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="164" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:14">
       <c r="A164">
         <v>124</v>
       </c>
@@ -9102,7 +9294,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="165" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:14">
       <c r="A165">
         <v>125</v>
       </c>
@@ -9131,7 +9323,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="166" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:14">
       <c r="A166">
         <v>126</v>
       </c>
@@ -9160,7 +9352,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="167" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:14">
       <c r="A167">
         <v>127</v>
       </c>
@@ -9189,7 +9381,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="168" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:14">
       <c r="A168">
         <v>128</v>
       </c>
@@ -9227,7 +9419,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="169" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:14">
       <c r="A169">
         <v>129</v>
       </c>
@@ -9256,7 +9448,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="170" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:14">
       <c r="A170">
         <v>130</v>
       </c>
@@ -9285,7 +9477,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="171" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:14">
       <c r="A171">
         <v>131</v>
       </c>
@@ -9314,7 +9506,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="172" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:14">
       <c r="A172">
         <v>132</v>
       </c>
@@ -9343,7 +9535,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="173" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:14">
       <c r="A173">
         <v>133</v>
       </c>
@@ -9372,7 +9564,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="174" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:14">
       <c r="A174">
         <v>134</v>
       </c>
@@ -9401,7 +9593,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="175" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:14">
       <c r="A175">
         <v>135</v>
       </c>
@@ -9430,7 +9622,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="176" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:14">
       <c r="A176">
         <v>136</v>
       </c>
@@ -9459,7 +9651,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="177" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:14">
       <c r="A177">
         <v>137</v>
       </c>
@@ -9488,7 +9680,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="178" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:14">
       <c r="A178">
         <v>138</v>
       </c>
@@ -9517,7 +9709,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="179" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:14">
       <c r="A179">
         <v>139</v>
       </c>
@@ -9546,7 +9738,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="180" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:14">
       <c r="A180">
         <v>140</v>
       </c>
@@ -9575,7 +9767,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="181" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:14">
       <c r="A181">
         <v>141</v>
       </c>
@@ -9619,7 +9811,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="182" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:14">
       <c r="A182">
         <v>142</v>
       </c>
@@ -9663,7 +9855,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="183" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:14">
       <c r="A183">
         <v>143</v>
       </c>
@@ -9692,7 +9884,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="184" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:14">
       <c r="A184">
         <v>144</v>
       </c>
@@ -9721,7 +9913,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="185" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:14">
       <c r="A185">
         <v>145</v>
       </c>
@@ -9750,7 +9942,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="186" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:14">
       <c r="A186">
         <v>146</v>
       </c>
@@ -9779,7 +9971,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="187" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:14">
       <c r="A187">
         <v>147</v>
       </c>
@@ -9808,7 +10000,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="188" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:14">
       <c r="A188">
         <v>148</v>
       </c>
@@ -9837,7 +10029,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="189" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:14">
       <c r="A189">
         <v>152</v>
       </c>
@@ -9866,7 +10058,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="190" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:14">
       <c r="A190">
         <v>153</v>
       </c>
@@ -9895,7 +10087,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="191" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:14">
       <c r="A191">
         <v>154</v>
       </c>
@@ -9924,7 +10116,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="192" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:14">
       <c r="A192">
         <v>155</v>
       </c>
@@ -9953,7 +10145,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="193" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:14">
       <c r="A193">
         <v>156</v>
       </c>
@@ -9982,7 +10174,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="194" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:14">
       <c r="A194">
         <v>157</v>
       </c>
@@ -10011,7 +10203,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="195" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:14">
       <c r="A195">
         <v>158</v>
       </c>
@@ -10040,7 +10232,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="196" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:14">
       <c r="A196">
         <v>159</v>
       </c>
@@ -10069,7 +10261,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="197" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:14">
       <c r="A197">
         <v>160</v>
       </c>
@@ -10107,7 +10299,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="198" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:14">
       <c r="A198">
         <v>161</v>
       </c>
@@ -10136,7 +10328,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="199" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:14">
       <c r="A199">
         <v>162</v>
       </c>
@@ -10180,7 +10372,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="200" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:14">
       <c r="A200">
         <v>163</v>
       </c>
@@ -10209,7 +10401,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="201" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:14">
       <c r="A201">
         <v>164</v>
       </c>
@@ -10253,7 +10445,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="202" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:14">
       <c r="A202">
         <v>165</v>
       </c>
@@ -10297,7 +10489,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="203" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:14">
       <c r="A203">
         <v>166</v>
       </c>
@@ -10338,7 +10530,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="204" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:14">
       <c r="A204">
         <v>167</v>
       </c>
@@ -10367,7 +10559,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="205" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:14">
       <c r="A205">
         <v>168</v>
       </c>
@@ -10396,7 +10588,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="206" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:14">
       <c r="A206">
         <v>192</v>
       </c>
@@ -10436,18 +10628,297 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5ADFFB9-3508-498E-BA9A-F449C470BB6D}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <dimension ref="A1:Q7"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col min="1" max="1" width="8.125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.75" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="6.5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.5" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="18.75" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:17">
+      <c r="A1" t="s">
+        <v>633</v>
+      </c>
+      <c r="B1" t="s">
+        <v>634</v>
+      </c>
+      <c r="C1" t="s">
+        <v>635</v>
+      </c>
+      <c r="D1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1" t="s">
+        <v>7</v>
+      </c>
+      <c r="H1" t="s">
+        <v>10</v>
+      </c>
+      <c r="I1" t="s">
+        <v>636</v>
+      </c>
+      <c r="J1" t="s">
+        <v>637</v>
+      </c>
+      <c r="K1" t="s">
+        <v>638</v>
+      </c>
+      <c r="L1" t="s">
+        <v>677</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17">
+      <c r="A2" t="s">
+        <v>667</v>
+      </c>
+      <c r="B2" t="s">
+        <v>639</v>
+      </c>
+      <c r="C2" t="s">
+        <v>640</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>668</v>
+      </c>
+      <c r="E2" t="s">
+        <v>622</v>
+      </c>
+      <c r="F2">
+        <v>10</v>
+      </c>
+      <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2" t="s">
+        <v>641</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>674</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>642</v>
+      </c>
+      <c r="K2" t="s">
+        <v>643</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>678</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>681</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17">
+      <c r="A3" t="s">
+        <v>667</v>
+      </c>
+      <c r="B3" t="s">
+        <v>639</v>
+      </c>
+      <c r="C3" t="s">
+        <v>640</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>669</v>
+      </c>
+      <c r="E3" t="s">
+        <v>644</v>
+      </c>
+      <c r="F3">
+        <v>1</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3" t="s">
+        <v>645</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>675</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>646</v>
+      </c>
+      <c r="K3" t="s">
+        <v>647</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17">
+      <c r="A4" t="s">
+        <v>667</v>
+      </c>
+      <c r="B4" t="s">
+        <v>648</v>
+      </c>
+      <c r="C4" t="s">
+        <v>649</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>670</v>
+      </c>
+      <c r="E4" t="s">
+        <v>650</v>
+      </c>
+      <c r="F4">
+        <v>1</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4" t="s">
+        <v>651</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>652</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>653</v>
+      </c>
+      <c r="K4" t="s">
+        <v>647</v>
+      </c>
+      <c r="L4" t="s">
+        <v>680</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17">
+      <c r="A5" t="s">
+        <v>667</v>
+      </c>
+      <c r="B5" t="s">
+        <v>648</v>
+      </c>
+      <c r="C5" t="s">
+        <v>649</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>671</v>
+      </c>
+      <c r="E5" t="s">
+        <v>654</v>
+      </c>
+      <c r="F5">
+        <v>1</v>
+      </c>
+      <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5" t="s">
+        <v>655</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>657</v>
+      </c>
+      <c r="K5" t="s">
+        <v>647</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17">
+      <c r="A6" t="s">
+        <v>667</v>
+      </c>
+      <c r="B6" t="s">
+        <v>648</v>
+      </c>
+      <c r="C6" t="s">
+        <v>649</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>672</v>
+      </c>
+      <c r="E6" t="s">
+        <v>658</v>
+      </c>
+      <c r="F6">
+        <v>1</v>
+      </c>
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6" t="s">
+        <v>659</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>660</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>661</v>
+      </c>
+      <c r="K6" t="s">
+        <v>647</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17">
+      <c r="A7" t="s">
+        <v>667</v>
+      </c>
+      <c r="B7" t="s">
+        <v>662</v>
+      </c>
+      <c r="C7" t="s">
+        <v>663</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>673</v>
+      </c>
+      <c r="E7" t="s">
+        <v>664</v>
+      </c>
+      <c r="F7" t="s">
+        <v>267</v>
+      </c>
+      <c r="G7">
+        <v>0</v>
+      </c>
+      <c r="H7" t="s">
+        <v>665</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>676</v>
+      </c>
+      <c r="J7" s="1" t="s">
+        <v>666</v>
+      </c>
+      <c r="K7" t="s">
+        <v>643</v>
+      </c>
+      <c r="L7" t="s">
+        <v>679</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
added bit_mask and get_bit functions to tinyexpr, added UDS DIDs from sniffing
</commit_message>
<xml_diff>
--- a/sw/firmware/OBDII-PIDs.xlsx
+++ b/sw/firmware/OBDII-PIDs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kubai\Documents\CAN-Sniffer\sw\firmware\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA833BB2-29C9-4D0D-ADCF-C0CBA790C86C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{795E70C6-0A90-4159-82EC-37C2F0D1C203}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{429A65A5-501F-4DDC-877A-2B2A6BFACDF8}"/>
+    <workbookView xWindow="1950" yWindow="1950" windowWidth="28800" windowHeight="15345" activeTab="1" xr2:uid="{429A65A5-501F-4DDC-877A-2B2A6BFACDF8}"/>
   </bookViews>
   <sheets>
     <sheet name="obd2-pid" sheetId="2" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1725" uniqueCount="682">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1889" uniqueCount="776">
   <si>
     <t>PID (dec)</t>
   </si>
@@ -2092,6 +2092,301 @@
   </si>
   <si>
     <t>https://gemini.google.com/share/4034399b676c</t>
+  </si>
+  <si>
+    <t>0x2609</t>
+  </si>
+  <si>
+    <t>Exterior temp</t>
+  </si>
+  <si>
+    <t>03 22 26 09 00 00 00 00</t>
+  </si>
+  <si>
+    <t>0x260C</t>
+  </si>
+  <si>
+    <t>Front Left Vent Temperature</t>
+  </si>
+  <si>
+    <t>03 22 26 0C 00 00 00 00</t>
+  </si>
+  <si>
+    <t>04 62 26 0C 4B AA AA AA</t>
+  </si>
+  <si>
+    <t>04 62 26 09 F6 AA AA AA</t>
+  </si>
+  <si>
+    <t>0x260D</t>
+  </si>
+  <si>
+    <t>Front Right Vent Temperature</t>
+  </si>
+  <si>
+    <t>04 62 26 0D 2D AA AA AA</t>
+  </si>
+  <si>
+    <t>03 22 26 0D 00 00 00 00</t>
+  </si>
+  <si>
+    <t>0x260E</t>
+  </si>
+  <si>
+    <t>03 22 26 0F 00 00 00 00</t>
+  </si>
+  <si>
+    <t>04 62 26 0F 5E AA AA AA</t>
+  </si>
+  <si>
+    <t>Front Right Foot Vent</t>
+  </si>
+  <si>
+    <t>Front Left Foot Vent</t>
+  </si>
+  <si>
+    <t>0x2610</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 03 22 26 10 00 00 00 00</t>
+  </si>
+  <si>
+    <t>04 62 26 10 5C AA AA AA</t>
+  </si>
+  <si>
+    <t>0x2614</t>
+  </si>
+  <si>
+    <t>Sun Intensity Left</t>
+  </si>
+  <si>
+    <t>04 62 26 14 03 AA AA AA</t>
+  </si>
+  <si>
+    <t>03 22 26 14 00 00 00 00</t>
+  </si>
+  <si>
+    <t>0x2615</t>
+  </si>
+  <si>
+    <t>Sun Intensity Right</t>
+  </si>
+  <si>
+    <t>03 22 26 15 00 00 00 00</t>
+  </si>
+  <si>
+    <t>04 62 26 15 0A AA AA AA</t>
+  </si>
+  <si>
+    <t>0x263F</t>
+  </si>
+  <si>
+    <t>03 22 26 3F 00 00 00 00</t>
+  </si>
+  <si>
+    <t>Time Since Ignition Off</t>
+  </si>
+  <si>
+    <t>04 62 26 3F 00 AA AA AA</t>
+  </si>
+  <si>
+    <t>Actual Value</t>
+  </si>
+  <si>
+    <t>0x2650</t>
+  </si>
+  <si>
+    <t>Engine Running and Ignition On time</t>
+  </si>
+  <si>
+    <t>03 22 26 50 00 00 00 00</t>
+  </si>
+  <si>
+    <t>05 62 26 50 36 74 AA AA</t>
+  </si>
+  <si>
+    <t>54s E and 116s I</t>
+  </si>
+  <si>
+    <t>0x2654</t>
+  </si>
+  <si>
+    <t>Heated Seat Stage Left</t>
+  </si>
+  <si>
+    <t>03 22 26 54 00 00 00 00</t>
+  </si>
+  <si>
+    <t>04 62 26 54 03 AA AA AA</t>
+  </si>
+  <si>
+    <t>0x2655</t>
+  </si>
+  <si>
+    <t>Heated Seat Stage Right</t>
+  </si>
+  <si>
+    <t>03 22 26 55 00 00 00 00</t>
+  </si>
+  <si>
+    <t>04 62 26 55 03 AA AA AA</t>
+  </si>
+  <si>
+    <t>0-off, 1-high beam, 2- flasher</t>
+  </si>
+  <si>
+    <t>03 22 1F 03 00 00 00 00</t>
+  </si>
+  <si>
+    <t>04 62 1F 03 00 AA AA AA</t>
+  </si>
+  <si>
+    <t>Horn</t>
+  </si>
+  <si>
+    <t>0x1F03</t>
+  </si>
+  <si>
+    <t>Windshield Wiper</t>
+  </si>
+  <si>
+    <t>03 22 1F 04 00 00 00 00</t>
+  </si>
+  <si>
+    <t>05 62 1F 04 80 01 AA AA</t>
+  </si>
+  <si>
+    <t>0x1F04</t>
+  </si>
+  <si>
+    <t>Byte 4
+0x01	Auto / Intermittent (Stalk Up 1 Position)
+0x02	Low Speed (Stalk Up 2 Positions)
+0x04	High Speed (Stalk Up 3 Positions)
+0x08	Flick / Mist (Stalk Pushed Down)
+0x10	Intermittent Stage 1 (Bottom)
+0x20	Intermittent Stage 2
+0x30	Intermittent Stage 3
+0x40	Intermittent Stage 4 (Top)
+0x80	Washer Pump Active
+Byte 5
+0x01	Motor Parked (Home)
+0x00	Motor in Motion</t>
+  </si>
+  <si>
+    <t>03 22 1F 05 00 00 00 00</t>
+  </si>
+  <si>
+    <t>04 62 1F 05 01 AA AA AA</t>
+  </si>
+  <si>
+    <t>0x04: Rear Washer Active (Pump spraying).
+0x01: Rear Wiper Active (Motor running/sweep).</t>
+  </si>
+  <si>
+    <t>Rear Wiper</t>
+  </si>
+  <si>
+    <t>03 22 22 20 00 00 00 00</t>
+  </si>
+  <si>
+    <t>Status of Input Signals</t>
+  </si>
+  <si>
+    <t>04 62 22 20 A5 AA AA AA</t>
+  </si>
+  <si>
+    <t>bitmask - parking brake active, insuffitient brake fluid not active, inssufitient washer active, insuffitient coolant not active, brake pad wear not active,</t>
+  </si>
+  <si>
+    <t>03 22 22 43 00 00 00 00</t>
+  </si>
+  <si>
+    <t>0x2220</t>
+  </si>
+  <si>
+    <t>05 62 22 43 00 61 AA AA</t>
+  </si>
+  <si>
+    <t>0x2243</t>
+  </si>
+  <si>
+    <t>Distance Driven from Inspection</t>
+  </si>
+  <si>
+    <t>9700km</t>
+  </si>
+  <si>
+    <t>03 22 22 44 00 00 00 00</t>
+  </si>
+  <si>
+    <t>05 62 22 44 00 F2 AA AA</t>
+  </si>
+  <si>
+    <t>Time Since Inspection</t>
+  </si>
+  <si>
+    <t>0x2244</t>
+  </si>
+  <si>
+    <t>03 22 22 48 00 00 00 00</t>
+  </si>
+  <si>
+    <t>04 62 22 48 01 AA AA AA</t>
+  </si>
+  <si>
+    <t>Oil quality</t>
+  </si>
+  <si>
+    <t>0x2248</t>
+  </si>
+  <si>
+    <t>poor, 0 good</t>
+  </si>
+  <si>
+    <t>Operating Range Calculated</t>
+  </si>
+  <si>
+    <t>05 62 22 94 01 93 AA AA</t>
+  </si>
+  <si>
+    <t>03 22 22 94 00 00 00 00</t>
+  </si>
+  <si>
+    <t>app shows 259, car 410, cloud be miles??</t>
+  </si>
+  <si>
+    <t>0x2294</t>
+  </si>
+  <si>
+    <t>Operating Range Fueld Consumption</t>
+  </si>
+  <si>
+    <t>car at stop 0,1</t>
+  </si>
+  <si>
+    <t>03 22 22 AB 00 00 00 00</t>
+  </si>
+  <si>
+    <t>04 62 22 AB 80 AA AA AA</t>
+  </si>
+  <si>
+    <t>0x22AB</t>
+  </si>
+  <si>
+    <t>Operating Range Fueld Supply</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 03 22 22 9A 00 00 00 00</t>
+  </si>
+  <si>
+    <t>05 62 22 9A 01 07 AA AA</t>
+  </si>
+  <si>
+    <t>0x229A</t>
+  </si>
+  <si>
+    <t>Battery Voltage</t>
   </si>
 </sst>
 </file>
@@ -2141,12 +2436,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normální" xfId="0" builtinId="0"/>
@@ -2245,9 +2541,9 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{4F04E350-6D47-4E09-A10B-E6A8E1D51955}" name="Tabulka2" displayName="Tabulka2" ref="A1:L7" totalsRowShown="0">
-  <autoFilter ref="A1:L7" xr:uid="{4F04E350-6D47-4E09-A10B-E6A8E1D51955}"/>
-  <tableColumns count="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{4F04E350-6D47-4E09-A10B-E6A8E1D51955}" name="Tabulka2" displayName="Tabulka2" ref="A1:M29" totalsRowShown="0">
+  <autoFilter ref="A1:M29" xr:uid="{4F04E350-6D47-4E09-A10B-E6A8E1D51955}"/>
+  <tableColumns count="13">
     <tableColumn id="1" xr3:uid="{984946A5-A725-4CB2-BED2-DAC7593D2235}" name="Car"/>
     <tableColumn id="2" xr3:uid="{9D892733-4D76-4C99-8DC4-07953415758A}" name="Module Name"/>
     <tableColumn id="3" xr3:uid="{10BD86BD-0BAD-4B7E-90DB-2D0150792BAC}" name="Module ID"/>
@@ -2260,6 +2556,7 @@
     <tableColumn id="10" xr3:uid="{AF2DE9E7-F7D7-40A7-B409-1C9D7BC25D21}" name="Example Response" dataDxfId="0"/>
     <tableColumn id="11" xr3:uid="{29F6CD0E-77A6-469F-94F0-37C29C2492CF}" name="Bit S|L"/>
     <tableColumn id="12" xr3:uid="{DF261B1A-8F21-48FD-902C-7E2E39B9973C}" name="Sloupec1"/>
+    <tableColumn id="13" xr3:uid="{81D60D28-9A44-4FAB-A360-936B66E209EA}" name="Actual Value"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -10637,7 +10934,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5ADFFB9-3508-498E-BA9A-F449C470BB6D}">
-  <dimension ref="A1:Q7"/>
+  <dimension ref="A1:Q29"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="8.125" bestFit="1" customWidth="1"/>
@@ -10648,8 +10945,9 @@
     <col min="6" max="6" width="7.75" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="8.375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="6.5" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18.5" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="18.75" customWidth="1"/>
+    <col min="9" max="9" width="24.625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="25.5" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17">
@@ -10689,6 +10987,9 @@
       <c r="L1" t="s">
         <v>677</v>
       </c>
+      <c r="M1" t="s">
+        <v>714</v>
+      </c>
     </row>
     <row r="2" spans="1:17">
       <c r="A2" t="s">
@@ -10838,6 +11139,9 @@
       <c r="K5" t="s">
         <v>647</v>
       </c>
+      <c r="M5" t="s">
+        <v>728</v>
+      </c>
     </row>
     <row r="6" spans="1:17">
       <c r="A6" t="s">
@@ -10910,6 +11214,575 @@
       </c>
       <c r="L7" t="s">
         <v>679</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17">
+      <c r="A8" t="s">
+        <v>667</v>
+      </c>
+      <c r="B8" t="s">
+        <v>662</v>
+      </c>
+      <c r="C8" t="s">
+        <v>663</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>682</v>
+      </c>
+      <c r="E8" t="s">
+        <v>683</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>684</v>
+      </c>
+      <c r="J8" s="1" t="s">
+        <v>689</v>
+      </c>
+      <c r="M8">
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17">
+      <c r="A9" t="s">
+        <v>667</v>
+      </c>
+      <c r="B9" t="s">
+        <v>662</v>
+      </c>
+      <c r="C9" t="s">
+        <v>663</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>685</v>
+      </c>
+      <c r="E9" t="s">
+        <v>686</v>
+      </c>
+      <c r="I9" s="1" t="s">
+        <v>687</v>
+      </c>
+      <c r="J9" s="1" t="s">
+        <v>688</v>
+      </c>
+      <c r="M9">
+        <v>25.7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17">
+      <c r="A10" t="s">
+        <v>667</v>
+      </c>
+      <c r="B10" t="s">
+        <v>662</v>
+      </c>
+      <c r="C10" t="s">
+        <v>663</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>690</v>
+      </c>
+      <c r="E10" t="s">
+        <v>691</v>
+      </c>
+      <c r="I10" s="1" t="s">
+        <v>693</v>
+      </c>
+      <c r="J10" s="1" t="s">
+        <v>692</v>
+      </c>
+      <c r="M10">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17">
+      <c r="A11" t="s">
+        <v>667</v>
+      </c>
+      <c r="B11" t="s">
+        <v>662</v>
+      </c>
+      <c r="C11" t="s">
+        <v>663</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>694</v>
+      </c>
+      <c r="E11" t="s">
+        <v>698</v>
+      </c>
+      <c r="I11" s="1" t="s">
+        <v>695</v>
+      </c>
+      <c r="J11" s="1" t="s">
+        <v>696</v>
+      </c>
+      <c r="M11">
+        <v>31.3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17">
+      <c r="A12" t="s">
+        <v>667</v>
+      </c>
+      <c r="B12" t="s">
+        <v>662</v>
+      </c>
+      <c r="C12" t="s">
+        <v>663</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>699</v>
+      </c>
+      <c r="E12" t="s">
+        <v>697</v>
+      </c>
+      <c r="I12" s="1" t="s">
+        <v>700</v>
+      </c>
+      <c r="J12" s="1" t="s">
+        <v>701</v>
+      </c>
+      <c r="M12">
+        <v>31.4</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17">
+      <c r="A13" t="s">
+        <v>667</v>
+      </c>
+      <c r="B13" t="s">
+        <v>662</v>
+      </c>
+      <c r="C13" t="s">
+        <v>663</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>702</v>
+      </c>
+      <c r="E13" t="s">
+        <v>703</v>
+      </c>
+      <c r="I13" s="1" t="s">
+        <v>705</v>
+      </c>
+      <c r="J13" s="1" t="s">
+        <v>704</v>
+      </c>
+      <c r="M13">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17">
+      <c r="A14" t="s">
+        <v>667</v>
+      </c>
+      <c r="B14" t="s">
+        <v>662</v>
+      </c>
+      <c r="C14" t="s">
+        <v>663</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>706</v>
+      </c>
+      <c r="E14" t="s">
+        <v>707</v>
+      </c>
+      <c r="I14" s="1" t="s">
+        <v>708</v>
+      </c>
+      <c r="J14" s="1" t="s">
+        <v>709</v>
+      </c>
+      <c r="M14">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="15" spans="1:17">
+      <c r="A15" t="s">
+        <v>667</v>
+      </c>
+      <c r="B15" t="s">
+        <v>662</v>
+      </c>
+      <c r="C15" t="s">
+        <v>663</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>710</v>
+      </c>
+      <c r="E15" t="s">
+        <v>712</v>
+      </c>
+      <c r="I15" s="1" t="s">
+        <v>711</v>
+      </c>
+      <c r="J15" s="1" t="s">
+        <v>713</v>
+      </c>
+      <c r="M15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17">
+      <c r="A16" t="s">
+        <v>667</v>
+      </c>
+      <c r="B16" t="s">
+        <v>662</v>
+      </c>
+      <c r="C16" t="s">
+        <v>663</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>715</v>
+      </c>
+      <c r="E16" t="s">
+        <v>716</v>
+      </c>
+      <c r="I16" s="1" t="s">
+        <v>717</v>
+      </c>
+      <c r="J16" s="1" t="s">
+        <v>718</v>
+      </c>
+      <c r="M16" t="s">
+        <v>719</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13">
+      <c r="A17" t="s">
+        <v>667</v>
+      </c>
+      <c r="B17" t="s">
+        <v>662</v>
+      </c>
+      <c r="C17" t="s">
+        <v>663</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>720</v>
+      </c>
+      <c r="E17" t="s">
+        <v>721</v>
+      </c>
+      <c r="I17" s="1" t="s">
+        <v>722</v>
+      </c>
+      <c r="J17" s="1" t="s">
+        <v>723</v>
+      </c>
+      <c r="M17">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13">
+      <c r="A18" t="s">
+        <v>667</v>
+      </c>
+      <c r="B18" t="s">
+        <v>662</v>
+      </c>
+      <c r="C18" t="s">
+        <v>663</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>724</v>
+      </c>
+      <c r="E18" t="s">
+        <v>725</v>
+      </c>
+      <c r="I18" s="1" t="s">
+        <v>726</v>
+      </c>
+      <c r="J18" s="1" t="s">
+        <v>727</v>
+      </c>
+      <c r="M18">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13">
+      <c r="A19" t="s">
+        <v>667</v>
+      </c>
+      <c r="B19" t="s">
+        <v>648</v>
+      </c>
+      <c r="C19" t="s">
+        <v>649</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>732</v>
+      </c>
+      <c r="E19" t="s">
+        <v>731</v>
+      </c>
+      <c r="I19" s="1" t="s">
+        <v>729</v>
+      </c>
+      <c r="J19" s="1" t="s">
+        <v>730</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13">
+      <c r="A20" t="s">
+        <v>667</v>
+      </c>
+      <c r="B20" t="s">
+        <v>648</v>
+      </c>
+      <c r="C20" t="s">
+        <v>649</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>736</v>
+      </c>
+      <c r="E20" t="s">
+        <v>733</v>
+      </c>
+      <c r="I20" s="1" t="s">
+        <v>734</v>
+      </c>
+      <c r="J20" s="1" t="s">
+        <v>735</v>
+      </c>
+      <c r="M20" s="3" t="s">
+        <v>737</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13">
+      <c r="A21" t="s">
+        <v>667</v>
+      </c>
+      <c r="B21" t="s">
+        <v>648</v>
+      </c>
+      <c r="C21" t="s">
+        <v>649</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>672</v>
+      </c>
+      <c r="E21" t="s">
+        <v>741</v>
+      </c>
+      <c r="I21" s="1" t="s">
+        <v>738</v>
+      </c>
+      <c r="J21" s="1" t="s">
+        <v>739</v>
+      </c>
+      <c r="M21" s="3" t="s">
+        <v>740</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13">
+      <c r="A22" t="s">
+        <v>667</v>
+      </c>
+      <c r="B22" t="s">
+        <v>639</v>
+      </c>
+      <c r="C22" t="s">
+        <v>640</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>747</v>
+      </c>
+      <c r="E22" t="s">
+        <v>743</v>
+      </c>
+      <c r="I22" s="1" t="s">
+        <v>742</v>
+      </c>
+      <c r="J22" s="1" t="s">
+        <v>744</v>
+      </c>
+      <c r="M22" t="s">
+        <v>745</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13">
+      <c r="A23" t="s">
+        <v>667</v>
+      </c>
+      <c r="B23" t="s">
+        <v>639</v>
+      </c>
+      <c r="C23" t="s">
+        <v>640</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>749</v>
+      </c>
+      <c r="E23" t="s">
+        <v>750</v>
+      </c>
+      <c r="I23" s="1" t="s">
+        <v>746</v>
+      </c>
+      <c r="J23" s="1" t="s">
+        <v>748</v>
+      </c>
+      <c r="M23" t="s">
+        <v>751</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13">
+      <c r="A24" t="s">
+        <v>667</v>
+      </c>
+      <c r="B24" t="s">
+        <v>639</v>
+      </c>
+      <c r="C24" t="s">
+        <v>640</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>755</v>
+      </c>
+      <c r="E24" t="s">
+        <v>754</v>
+      </c>
+      <c r="I24" s="1" t="s">
+        <v>752</v>
+      </c>
+      <c r="J24" s="1" t="s">
+        <v>753</v>
+      </c>
+      <c r="M24">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13">
+      <c r="A25" t="s">
+        <v>667</v>
+      </c>
+      <c r="B25" t="s">
+        <v>639</v>
+      </c>
+      <c r="C25" t="s">
+        <v>640</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>759</v>
+      </c>
+      <c r="E25" t="s">
+        <v>758</v>
+      </c>
+      <c r="I25" s="1" t="s">
+        <v>756</v>
+      </c>
+      <c r="J25" s="1" t="s">
+        <v>757</v>
+      </c>
+      <c r="M25" t="s">
+        <v>760</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13">
+      <c r="A26" t="s">
+        <v>667</v>
+      </c>
+      <c r="B26" t="s">
+        <v>639</v>
+      </c>
+      <c r="C26" t="s">
+        <v>640</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>765</v>
+      </c>
+      <c r="E26" t="s">
+        <v>761</v>
+      </c>
+      <c r="I26" s="1" t="s">
+        <v>763</v>
+      </c>
+      <c r="J26" s="1" t="s">
+        <v>762</v>
+      </c>
+      <c r="M26" t="s">
+        <v>764</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13">
+      <c r="A27" t="s">
+        <v>667</v>
+      </c>
+      <c r="B27" t="s">
+        <v>639</v>
+      </c>
+      <c r="C27" t="s">
+        <v>640</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>765</v>
+      </c>
+      <c r="E27" t="s">
+        <v>766</v>
+      </c>
+      <c r="I27" s="1" t="s">
+        <v>763</v>
+      </c>
+      <c r="J27" s="1" t="s">
+        <v>762</v>
+      </c>
+      <c r="M27" t="s">
+        <v>767</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13">
+      <c r="A28" t="s">
+        <v>667</v>
+      </c>
+      <c r="B28" t="s">
+        <v>639</v>
+      </c>
+      <c r="C28" t="s">
+        <v>640</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>770</v>
+      </c>
+      <c r="E28" t="s">
+        <v>771</v>
+      </c>
+      <c r="I28" s="1" t="s">
+        <v>768</v>
+      </c>
+      <c r="J28" s="1" t="s">
+        <v>769</v>
+      </c>
+      <c r="M28">
+        <v>32.875</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13">
+      <c r="A29" t="s">
+        <v>667</v>
+      </c>
+      <c r="B29" t="s">
+        <v>639</v>
+      </c>
+      <c r="C29" t="s">
+        <v>640</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>774</v>
+      </c>
+      <c r="E29" t="s">
+        <v>775</v>
+      </c>
+      <c r="I29" s="1" t="s">
+        <v>772</v>
+      </c>
+      <c r="J29" s="1" t="s">
+        <v>773</v>
+      </c>
+      <c r="M29">
+        <v>12.03</v>
       </c>
     </row>
   </sheetData>

</xml_diff>